<commit_message>
adding sal B and its two domains to the dataset. Also changed code in layer2 so it goes into the structures folder and structures dont need to be brought into same directory
</commit_message>
<xml_diff>
--- a/494/initial.xlsx
+++ b/494/initial.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jpwillms\Desktop\LocalCode\494\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jpwillms\Desktop\494\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4355848B-F6CD-4AB4-A7B1-8D00C827C03F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C196EC0-5B4D-45DF-ABF2-C7F23887907D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="30975" yWindow="2760" windowWidth="21600" windowHeight="11295" xr2:uid="{92F93940-16D1-494E-8DAD-2FEDD2E887ED}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{92F93940-16D1-494E-8DAD-2FEDD2E887ED}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="476" uniqueCount="333">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="494" uniqueCount="344">
   <si>
     <t>Source</t>
   </si>
@@ -1038,13 +1038,46 @@
   </si>
   <si>
     <t>JP_d1</t>
+  </si>
+  <si>
+    <t>H7C6X6</t>
+  </si>
+  <si>
+    <t>Enterococcus faecalis</t>
+  </si>
+  <si>
+    <t>SalB</t>
+  </si>
+  <si>
+    <t>SalB domain 1 (long)</t>
+  </si>
+  <si>
+    <t>SalB domain 2 (globular)</t>
+  </si>
+  <si>
+    <t>MKKRLFASVLLCSLTLSAIATPSIALADNVDKKIEEKNQEISSLKAKQGDLASQVSSLEA EVSSVFDESMALREQKQTLKAKSEQLQQEITNLNQRIEKRNEAIKNQARDVQVNGQSTTM LDAVLDADSVADAISRVQAVSTIVSANNDLMQQQKEDKQAVVDKKAENEKKVKQLEATEA ELETKRQDLLSKQSELNVMKASLALEQSSAESSKAGLEKQKAAAEAEQARLAAEQKAAAE KAKQAAAKPAKAEVKAEAPVASSSTTEAQAPASSSSATESSTQQTTETTTPSTDNSATEN TGSSSSEQPVQPTTPSDNGNNGGQTGGGTVTPTPEPTPAPSADPTINALNVLRQSLGLRP VVWDAGLAASATARAAQVEAGGIPNDHWSRGDEVIAIMWAPGNSVIMAWYNETNMVTASG SGHRDWEINPGITRVGFGYSGSTIVGHSA</t>
+  </si>
+  <si>
+    <t>SIALADNVDKKIEEKNQEISSLKAKQGDLASQVSSLEA EVSSVFDESMALREQKQTLKAKSEQLQQEITNLNQRIEKRNEAIKNQARDVQVNGQSTTM LDAVLDADSVADAISRVQAVSTIVSANNDLMQQQKEDKQAVVDKKAENEKKVKQLEATEA ELETKRQDLLSKQSELNVMKASLALEQSSAESSKAGLEKQKAAAEAEQARLAAEQKAAAE KAKQAAAKPA</t>
+  </si>
+  <si>
+    <t>ADPTINALNVLRQSLGLRP VVWDAGLAASATARAAQVEAGGIPNDHWSRGDEVIAIMWAPGNSVIMAWYNETNMVTASG SGHRDWEINPGITRVGFGYSGSTIVGHSA</t>
+  </si>
+  <si>
+    <t>AF-H7C6X6-F1</t>
+  </si>
+  <si>
+    <t>Sal_d1</t>
+  </si>
+  <si>
+    <t>Sal_d2</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1087,6 +1120,13 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color rgb="FF0A0A0A"/>
+      <name val="Lato"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="7">
@@ -1155,7 +1195,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -1193,6 +1233,7 @@
     <xf numFmtId="0" fontId="6" fillId="6" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -3599,35 +3640,83 @@
         <v>331</v>
       </c>
     </row>
-    <row r="81" spans="1:8" ht="15.75" thickBot="1">
-      <c r="A81" s="1"/>
-      <c r="B81" s="1"/>
-      <c r="C81" s="1"/>
-      <c r="D81" s="1"/>
-      <c r="E81" s="1"/>
-      <c r="F81" s="1"/>
-      <c r="G81" s="1"/>
-      <c r="H81" s="1"/>
-    </row>
-    <row r="82" spans="1:8" ht="15.75" thickBot="1">
-      <c r="A82" s="1"/>
-      <c r="B82" s="1"/>
-      <c r="C82" s="1"/>
-      <c r="D82" s="1"/>
-      <c r="E82" s="1"/>
-      <c r="F82" s="1"/>
-      <c r="G82" s="1"/>
-      <c r="H82" s="1"/>
-    </row>
-    <row r="83" spans="1:8" ht="15.75" thickBot="1">
-      <c r="A83" s="1"/>
-      <c r="B83" s="1"/>
-      <c r="C83" s="1"/>
-      <c r="D83" s="1"/>
-      <c r="E83" s="1"/>
-      <c r="F83" s="1"/>
-      <c r="G83" s="1"/>
-      <c r="H83" s="1"/>
+    <row r="81" spans="1:8" ht="39.75" thickBot="1">
+      <c r="A81" s="13" t="s">
+        <v>333</v>
+      </c>
+      <c r="B81" s="1" t="s">
+        <v>334</v>
+      </c>
+      <c r="C81" s="1" t="s">
+        <v>335</v>
+      </c>
+      <c r="D81" t="s">
+        <v>11</v>
+      </c>
+      <c r="E81" t="s">
+        <v>338</v>
+      </c>
+      <c r="F81" s="1">
+        <v>0</v>
+      </c>
+      <c r="G81" s="1">
+        <v>80</v>
+      </c>
+      <c r="H81" s="1" t="s">
+        <v>341</v>
+      </c>
+    </row>
+    <row r="82" spans="1:8" ht="39.75" thickBot="1">
+      <c r="A82" s="13" t="s">
+        <v>333</v>
+      </c>
+      <c r="B82" s="1" t="s">
+        <v>334</v>
+      </c>
+      <c r="C82" s="1" t="s">
+        <v>336</v>
+      </c>
+      <c r="D82" t="s">
+        <v>11</v>
+      </c>
+      <c r="E82" t="s">
+        <v>339</v>
+      </c>
+      <c r="F82" s="1">
+        <v>0</v>
+      </c>
+      <c r="G82" s="1">
+        <v>81</v>
+      </c>
+      <c r="H82" s="1" t="s">
+        <v>342</v>
+      </c>
+    </row>
+    <row r="83" spans="1:8" ht="39.75" thickBot="1">
+      <c r="A83" s="13" t="s">
+        <v>333</v>
+      </c>
+      <c r="B83" s="1" t="s">
+        <v>334</v>
+      </c>
+      <c r="C83" s="1" t="s">
+        <v>337</v>
+      </c>
+      <c r="D83" t="s">
+        <v>11</v>
+      </c>
+      <c r="E83" t="s">
+        <v>340</v>
+      </c>
+      <c r="F83" s="1">
+        <v>0</v>
+      </c>
+      <c r="G83" s="1">
+        <v>82</v>
+      </c>
+      <c r="H83" s="1" t="s">
+        <v>343</v>
+      </c>
     </row>
     <row r="84" spans="1:8" ht="15.75" thickBot="1">
       <c r="A84" s="1"/>
@@ -12035,6 +12124,7 @@
     <hyperlink ref="C78" r:id="rId62" display="https://www.ebi.ac.uk/interpro/protein/reviewed/C0H3T3/" xr:uid="{2FA58E87-4E9F-4DFC-90E7-38A1D6FBC6DF}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId63"/>
 </worksheet>
 </file>
 

</xml_diff>